<commit_message>
chore: publish acknowledgement IG 2.0.3
</commit_message>
<xml_diff>
--- a/ig/acknowledgement/StructureDefinition-medcom-acknowledgement-operationoutcome.xlsx
+++ b/ig/acknowledgement/StructureDefinition-medcom-acknowledgement-operationoutcome.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.2</t>
+    <t>2.0.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-05T12:26:02+01:00</t>
+    <t>2026-02-05T13:48:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -69,7 +69,7 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>No display for ContactDetail</t>
+    <t>MedCom (http://www.medcom.dk)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
@@ -355,7 +355,7 @@
     <t>A human language.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/languages</t>
+    <t>http://hl7.org/fhir/ValueSet/languages|4.0.1</t>
   </si>
   <si>
     <t>Resource.language</t>
@@ -597,7 +597,7 @@
     <t>A code that provides details as the exact issue.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/operation-outcome</t>
+    <t>http://hl7.org/fhir/ValueSet/operation-outcome|4.0.1</t>
   </si>
   <si>
     <t>ERR-5</t>
@@ -1041,17 +1041,17 @@
   <dimension ref="A1:AL24"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="40.3125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="40.3125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.1328125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="38.81640625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.90234375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.69921875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="5.07421875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="14.625" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.98828125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="35.17578125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="35.17578125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="17.203125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="15.140625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1060,24 +1060,24 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.84375" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="15.71484375" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="16.08984375" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="17.078125" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="16.3125" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="43.19921875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="81.2578125" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.69140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.73046875" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="40.0390625" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="14.98828125" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="12.3046875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="34.0703125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="9.5" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="9.87890625" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="8.53515625" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="38.43359375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="69.94140625" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="29.88671875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="245.55859375" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="43.93359375" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="217.1875" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="39.109375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2168,7 +2168,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" hidden="true">
+    <row r="11">
       <c r="A11" t="s" s="2">
         <v>141</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" hidden="true">
+    <row r="15">
       <c r="A15" t="s" s="2">
         <v>161</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="16" hidden="true">
+    <row r="16">
       <c r="A16" t="s" s="2">
         <v>171</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="17" hidden="true">
+    <row r="17">
       <c r="A17" t="s" s="2">
         <v>179</v>
       </c>
@@ -3138,7 +3138,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" hidden="true">
+    <row r="20">
       <c r="A20" t="s" s="2">
         <v>193</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="21" hidden="true">
+    <row r="21">
       <c r="A21" t="s" s="2">
         <v>203</v>
       </c>
@@ -3686,12 +3686,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AL24">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
chore: publish acknowledgement IG 2.0.3 (#63)
Co-authored-by: tmsMedcom <tmsMedcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/acknowledgement/StructureDefinition-medcom-acknowledgement-operationoutcome.xlsx
+++ b/ig/acknowledgement/StructureDefinition-medcom-acknowledgement-operationoutcome.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.2</t>
+    <t>2.0.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-05T12:26:02+01:00</t>
+    <t>2026-02-05T13:48:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -69,7 +69,7 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>No display for ContactDetail</t>
+    <t>MedCom (http://www.medcom.dk)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
@@ -355,7 +355,7 @@
     <t>A human language.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/languages</t>
+    <t>http://hl7.org/fhir/ValueSet/languages|4.0.1</t>
   </si>
   <si>
     <t>Resource.language</t>
@@ -597,7 +597,7 @@
     <t>A code that provides details as the exact issue.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/operation-outcome</t>
+    <t>http://hl7.org/fhir/ValueSet/operation-outcome|4.0.1</t>
   </si>
   <si>
     <t>ERR-5</t>
@@ -1041,17 +1041,17 @@
   <dimension ref="A1:AL24"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="40.3125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="40.3125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.1328125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="38.81640625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.90234375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.69921875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="5.07421875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="14.625" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.98828125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="35.17578125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="35.17578125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="17.203125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="15.140625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1060,24 +1060,24 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.84375" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="15.71484375" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="16.08984375" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="17.078125" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="16.3125" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="43.19921875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="81.2578125" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.69140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.73046875" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="40.0390625" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="14.98828125" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="12.3046875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="34.0703125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="9.5" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="9.87890625" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="8.53515625" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="38.43359375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="69.94140625" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="29.88671875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="245.55859375" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="43.93359375" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="217.1875" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="39.109375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2168,7 +2168,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" hidden="true">
+    <row r="11">
       <c r="A11" t="s" s="2">
         <v>141</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" hidden="true">
+    <row r="15">
       <c r="A15" t="s" s="2">
         <v>161</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="16" hidden="true">
+    <row r="16">
       <c r="A16" t="s" s="2">
         <v>171</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="17" hidden="true">
+    <row r="17">
       <c r="A17" t="s" s="2">
         <v>179</v>
       </c>
@@ -3138,7 +3138,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" hidden="true">
+    <row r="20">
       <c r="A20" t="s" s="2">
         <v>193</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="21" hidden="true">
+    <row r="21">
       <c r="A21" t="s" s="2">
         <v>203</v>
       </c>
@@ -3686,12 +3686,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AL24">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>